<commit_message>
feat(rxkids): add optional 12-month postnatal extension as a "potential" line
Base run keeps the 6-month postnatal window. The cost output now also
prices the optional extension to the full 12 months (Flint upper bound)
as a clearly-labeled "POTENTIAL" add-on — additional +6-month cost and the
resulting 12-month total — in the workbook Summary, the PDF, and the state
CSV (potential_additional_6mo_cost_$, potential_total_12mo_cost_$). The
program may or may not opt in.

Real-PUMS TY2028: base $52.5M; +6 months +$16.1M; 12-month total $68.7M.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
+++ b/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -591,55 +591,85 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>HOUSEHOLD REACH</t>
+          <t>POTENTIAL — extend postnatal 6→12 months (optional)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Families reached (weighted)</t>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Additional cost (+6 months)</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>306411</v>
+        <v>16148563.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Total cost (12-month design)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>68693606.40000001</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>HOUSEHOLD REACH</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Families reached (weighted)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>306411</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Prenatal (expectant filers)</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B20" s="5" t="n">
         <v>245248</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Postnatal (families w/ infants)</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B21" s="5" t="n">
         <v>96130</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Avg benefit per family reached</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B22" s="5" t="n">
         <v>171.4854988887475</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Benefits by income quintile → see the 'By income quintile' tab.</t>
         </is>
@@ -1213,7 +1243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1262,7 +1292,7 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Caveats: 2026-2028 FPL is CPI-projected off the 2025 HHS table; pregnancy incidence and infant share are held at base-year values.</t>
+          <t>The base run prices the 6-month postnatal window (Flint's lower bound). The 'potential' line prices the optional extension to the full 12 months — the program may or may not opt in. Postnatal cost is linear in months, so the additional 6 months roughly equals the base postnatal arm again.</t>
         </is>
       </c>
     </row>
@@ -1271,6 +1301,16 @@
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Caveats: 2026-2028 FPL is CPI-projected off the 2025 HHS table; pregnancy incidence and infant share are held at base-year values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Full methodology: RXKIDS_METHODOLOGY.md (program origin, parameter sourcing, eligibility approximations, limitations).</t>
         </is>

</xml_diff>

<commit_message>
feat(rxkids): raise default take-up 0.80 -> 0.90
Default take-up_rate is now 0.90 (still below Flint's observed 0.98 to reflect
weaker year-1 Hawaii infrastructure). Updated the dataclass default, the
forecast CLI default, the factory test, and the docs. Conservative headline
moves ~$41M -> ~$46M (prenatal ~$15M + postnatal ~$31M); band ~$28M-$59M.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
+++ b/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>40954399.2</v>
+        <v>46073699.10000001</v>
       </c>
     </row>
     <row r="6">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>13651466.4</v>
+        <v>15357899.7</v>
       </c>
     </row>
     <row r="7">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>27302932.8</v>
+        <v>30715799.40000001</v>
       </c>
     </row>
     <row r="8">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>37989529.63650627</v>
+        <v>42738220.84106956</v>
       </c>
     </row>
     <row r="9">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>43919268.76349373</v>
+        <v>49409177.35893046</v>
       </c>
     </row>
     <row r="10">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>1802352.318233272</v>
+        <v>2027646.358012431</v>
       </c>
     </row>
     <row r="11">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>23036849.55</v>
+        <v>27644219.46</v>
       </c>
     </row>
     <row r="12">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>60791686.3125</v>
+        <v>58743966.35250001</v>
       </c>
     </row>
     <row r="13">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>27302932.8</v>
+        <v>30715799.39999999</v>
       </c>
     </row>
     <row r="16">
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>68257332</v>
+        <v>76789498.5</v>
       </c>
     </row>
     <row r="17">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>17127534.23333333</v>
+        <v>19268476.0125</v>
       </c>
     </row>
     <row r="20">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>7394544.3</v>
+        <v>8318862.337499999</v>
       </c>
     </row>
     <row r="21">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>9732989.933333334</v>
+        <v>10949613.675</v>
       </c>
     </row>
     <row r="22">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>5056098.66666667</v>
+        <v>5688111</v>
       </c>
     </row>
     <row r="23">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>26734121.7</v>
+        <v>30075886.9125</v>
       </c>
     </row>
     <row r="25">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>11418356.15555556</v>
+        <v>12845650.675</v>
       </c>
     </row>
     <row r="26">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>18201.9552</v>
+        <v>20477.1996</v>
       </c>
     </row>
     <row r="30">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>9100.977600000002</v>
+        <v>10238.5998</v>
       </c>
     </row>
     <row r="31">
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>9100.9776</v>
+        <v>10238.5998</v>
       </c>
     </row>
     <row r="32">
@@ -852,10 +852,10 @@
         <v>109745</v>
       </c>
       <c r="D2" s="11" t="n">
-        <v>5584</v>
+        <v>6281</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>11293145</v>
+        <v>12704789</v>
       </c>
       <c r="F2" s="11" t="n">
         <v>2023</v>
@@ -877,10 +877,10 @@
         <v>109845</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>6090</v>
+        <v>6852</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>13146650</v>
+        <v>14789981</v>
       </c>
       <c r="F3" s="11" t="n">
         <v>2159</v>
@@ -902,10 +902,10 @@
         <v>109868</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>4270</v>
+        <v>4803</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>10864331</v>
+        <v>12222373</v>
       </c>
       <c r="F4" s="11" t="n">
         <v>2545</v>
@@ -927,10 +927,10 @@
         <v>109862</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>1932</v>
+        <v>2173</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>4946859</v>
+        <v>5565216</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>2561</v>
@@ -952,10 +952,10 @@
         <v>109855</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>327</v>
+        <v>367</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>703413</v>
+        <v>791340</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>2154</v>
@@ -1025,19 +1025,19 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>8015434</v>
+        <v>9017363</v>
       </c>
       <c r="C2" s="11" t="n">
-        <v>2518003</v>
+        <v>2832754</v>
       </c>
       <c r="D2" s="11" t="n">
-        <v>5497430</v>
+        <v>6184609</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>791042</v>
+        <v>889923</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>3511</v>
+        <v>3950</v>
       </c>
     </row>
     <row r="3">
@@ -1047,19 +1047,19 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>26818793</v>
+        <v>30171142</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>9168756</v>
+        <v>10314851</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>17650037</v>
+        <v>19856291</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>1352049</v>
+        <v>1521055</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>11996</v>
+        <v>13495</v>
       </c>
     </row>
     <row r="4">
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>1703381</v>
+        <v>1916303</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>545794</v>
+        <v>614018</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>1157587</v>
+        <v>1302286</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>315863</v>
+        <v>355346</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>750</v>
+        <v>843</v>
       </c>
     </row>
     <row r="5">
@@ -1091,19 +1091,19 @@
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>4416792</v>
+        <v>4968890</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1418913</v>
+        <v>1596277</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>2997878</v>
+        <v>3372613</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>532342</v>
+        <v>598884</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>1945</v>
+        <v>2188</v>
       </c>
     </row>
   </sheetData>
@@ -1117,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1232,105 +1232,122 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Swept [0.6, 0.95] for the band</t>
+          <t>Combined eligibility×claim (Flint observed 0.98); swept for the band</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pregnancy probability (anchored)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.0521</v>
+          <t>Fertility response</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>+0%</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Birth-anchored from raw 0.1 so expected pregnancies = eligible births; swept ±25%</t>
+          <t>Induced eligible-birth increase (Flint ~+10%); scales both arms</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Child-under-age share</t>
+          <t>Pregnancy probability (anchored)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.066</v>
+        <v>0.0521</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Annual births ÷ dependents (FLOW); postnatal infant proxy; swept ±25%</t>
+          <t>Birth-anchored from raw 0.1 so expected pregnancies = eligible births; swept ±25%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FPL table year</t>
+          <t>Child-under-age share</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2028</v>
+        <v>0.066</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>benefits/_fpl.py (2025 published; 2026-28 CPI-projected)</t>
+          <t>Annual births ÷ dependents (FLOW); postnatal infant proxy; swept ±25%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tax treatment</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>non-taxable</t>
-        </is>
+          <t>FPL table year</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2028</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Added to SPM resources only; no AGI/EITC/CTC interaction</t>
+          <t>benefits/_fpl.py (2025 published; 2026-28 CPI-projected)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fiscal weight</t>
+          <t>Tax treatment</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>WGTP (household)</t>
+          <t>non-taxable</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SPM-grain household weight; not the EITC-reweighted tax-unit weight</t>
+          <t>Added to SPM resources only; no AGI/EITC/CTC interaction</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Fiscal weight</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>WGTP (household)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SPM-grain household weight; not the EITC-reweighted tax-unit weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Income quintiles</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>WGTP-weighted</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>SPM units ranked on summed income; population-equal fifths</t>
         </is>

</xml_diff>

<commit_message>
feat(rxkids): test eligibility on a MAGI proxy, not gross cash income
Medicaid/CHIP and ACA test eligibility on Modified Adjusted Gross Income.
The model's `income` counts only the 85% taxable portion of Social Security;
MAGI counts 100%. _magi_proxy adds back the non-taxable SS (ssp_full − ssp)
for both filers, and _attach_family_grain now sums MAGI (not gross income)
across the SPM family for both eligibility clauses. Above-the-line deductions
and tax-exempt interest are not observable in PUMS, so MAGI ≈ gross + SS
add-back (a standard survey-based proxy).

Effect (real PUMS TY2028): cost $46.07M -> $45.44M (-1.4%) — counting full SS
pushes some multigenerational families (grandparent on SS living with kids)
over 300% FPL. Retires the "wrong income object" caveat. Adds a unit test;
full suite (minus external) 1558 pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
+++ b/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>46073699.1</v>
+        <v>45436188.60000001</v>
       </c>
     </row>
     <row r="6">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>15357899.7</v>
+        <v>15145396.2</v>
       </c>
     </row>
     <row r="7">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>30715799.40000001</v>
+        <v>30290792.4</v>
       </c>
     </row>
     <row r="8">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>41600377.16850201</v>
+        <v>41009667.03018691</v>
       </c>
     </row>
     <row r="9">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>50547021.03149799</v>
+        <v>49862710.16981311</v>
       </c>
     </row>
     <row r="10">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>2719344.639208504</v>
+        <v>2690894.571314957</v>
       </c>
     </row>
     <row r="11">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>27644219.46</v>
+        <v>27261713.16</v>
       </c>
     </row>
     <row r="12">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>58743966.35250001</v>
+        <v>57931140.465</v>
       </c>
     </row>
     <row r="13">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>30715799.4</v>
+        <v>30290792.39999999</v>
       </c>
     </row>
     <row r="16">
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>76789498.5</v>
+        <v>75726981</v>
       </c>
     </row>
     <row r="17">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>19268476.0125</v>
+        <v>19001862.825</v>
       </c>
     </row>
     <row r="20">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>8318862.337500001</v>
+        <v>8203756.275</v>
       </c>
     </row>
     <row r="21">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>10949613.675</v>
+        <v>10798106.55</v>
       </c>
     </row>
     <row r="22">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>5688111</v>
+        <v>5609406.000000002</v>
       </c>
     </row>
     <row r="23">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>30075886.91250001</v>
+        <v>29659734.22499999</v>
       </c>
     </row>
     <row r="25">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>12845650.675</v>
+        <v>12667908.55</v>
       </c>
     </row>
     <row r="26">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>80867</v>
+        <v>79842</v>
       </c>
     </row>
     <row r="29">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>20477.1996</v>
+        <v>20193.8616</v>
       </c>
     </row>
     <row r="30">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>10238.5998</v>
+        <v>10096.9308</v>
       </c>
     </row>
     <row r="31">
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>10238.5998</v>
+        <v>10096.9308</v>
       </c>
     </row>
     <row r="32">
@@ -861,7 +861,7 @@
         <v>2250</v>
       </c>
       <c r="G2" s="12" t="n">
-        <v>21.4</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="3">
@@ -886,7 +886,7 @@
         <v>2250</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>29.4</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="4">
@@ -902,16 +902,16 @@
         <v>109868</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>6690</v>
+        <v>6636</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>15052198</v>
+        <v>14930309</v>
       </c>
       <c r="F4" s="11" t="n">
         <v>2250</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>32.7</v>
+        <v>32.9</v>
       </c>
     </row>
     <row r="5">
@@ -927,16 +927,16 @@
         <v>109862</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>3074</v>
+        <v>2952</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>6915586</v>
+        <v>6642138</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>2250</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>15</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="6">
@@ -952,16 +952,16 @@
         <v>109855</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>320</v>
+        <v>213</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>720641</v>
+        <v>478467</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>2250</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
     </row>
   </sheetData>
@@ -1025,19 +1025,19 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>9276914</v>
+        <v>9211693</v>
       </c>
       <c r="C2" s="11" t="n">
-        <v>3092305</v>
+        <v>3070564</v>
       </c>
       <c r="D2" s="11" t="n">
-        <v>6184609</v>
+        <v>6141128</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>1267084</v>
+        <v>1257092</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>4123</v>
+        <v>4094</v>
       </c>
     </row>
     <row r="3">
@@ -1047,19 +1047,19 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>29784437</v>
+        <v>29212148</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>9928146</v>
+        <v>9737383</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>19856291</v>
+        <v>19474765</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>2017916</v>
+        <v>2025493</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>13238</v>
+        <v>12983</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
fix(rxkids): correct stale PDF/workbook footnotes + fix PDF label clipping
The PDF footer and workbook Notes still described the old model (pregnancy-
probability adjustment, pregnancy-incidence in the band, SPM-unit eligibility
grain). Updated both to the current model: birth-event-driven arms, MAGI at
the tax-unit / MAGI-household eligibility grain, and a take-up + birth-rate
assumption band.

Also fixed a layout bug: a preceding multi_cell left the PDF cursor at the
right margin, clipping the next section's first label ("Addi…", "Year-…").
section()/kv() now reset x to the left margin. Verified both pages of the
conservative and Flint PDFs render with no clipping/overflow. Reports
regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
+++ b/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
@@ -1351,7 +1351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1370,7 +1370,7 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Cost = Σ (expected RxKids benefit × household weight) at SPM-unit grain. The benefit is already take-up- and pregnancy-probability-adjusted, so it is an expected annual dollar amount per unit, not a literal payment.</t>
+          <t>Both arms are driven by birth events (num_dependents × the annual birth rate per dependent); each eligible birth draws one prenatal + one postnatal payment. Cost = the take-up-adjusted benefit weighted by the household (WGTP) weight, summed to SPM-unit grain. Per-unit amounts are expectations, not literal payments.</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>Household impact here is the distribution of RxKids benefits RECEIVED across weighted income quintiles (SPM units ranked on summed income). This view does not use the tax engine or SPM poverty thresholds, so the whole run is genuine TY2028. A poverty-lift view (persons lifted) would require those engines, which stop at TY2025 — out of scope for this run.</t>
+          <t>Eligibility is tested on MAGI (gross income with 100% of Social Security) at the tax-unit / MAGI-household grain — the family Medicaid defines (42 CFR 435.603) — consistent with the statute's clause-1 Medicaid anchor. If the bill defines 'family' more broadly, the SPM-family grain (~$45M) is the alternative.</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1390,7 @@
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>Sampling 90% CI is ACS sampling error only (SDR over 80 PUMS replicate weights). The assumption band is a one-at-a-time sweep over the three soft, unanchored parameters (take-up, pregnancy incidence, infant share) — cost is linear in each.</t>
+          <t>Household impact here is the distribution of RxKids benefits RECEIVED across weighted income quintiles (SPM units ranked on summed income). This view does not use the tax engine or SPM poverty thresholds, so the whole run is genuine TY2028. A poverty-lift view (persons lifted) would require those engines, which stop at TY2025 — out of scope for this run.</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>The base run prices the 6-month postnatal window (Flint's lower bound). The 'potential' line prices the optional extension to the full 12 months — the program may or may not opt in. Postnatal cost is linear in months, so the additional 6 months roughly equals the base postnatal arm again.</t>
+          <t>Sampling 90% CI is ACS sampling error only (SDR over 80 PUMS replicate weights). The assumption band is the joint (all-low/all-high corner) sweep over the two soft, unanchored drivers — take-up and the birth rate — cost is linear in each.</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>Caveats: 2026-2028 FPL is CPI-projected off the 2025 HHS table; pregnancy incidence and infant share are held at base-year values.</t>
+          <t>The base run prices the 6-month postnatal window (Flint's lower bound). The 'potential' line prices the optional extension to the full 12 months — the program may or may not opt in. Postnatal cost is linear in months, so the additional 6 months roughly equals the base postnatal arm again.</t>
         </is>
       </c>
     </row>
@@ -1419,6 +1419,16 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Caveats: 2026-2028 FPL is CPI-projected off the 2025 HHS table; the birth rate is held at the base-year value (no 2028 birth-trend adjustment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Full methodology: RXKIDS_METHODOLOGY.md (program origin, parameter sourcing, eligibility approximations, limitations).</t>
         </is>

</xml_diff>

<commit_message>
feat(rxkids): arm-specific take-up (prenatal < postnatal per Flint evidence)
The literature shows mothers enroll prenatally at a lower rate than newborns
are enrolled (Flint: ~90% prenatal vs ~98% of newborns). Added
prenatal_takeup_rate: the postnatal/newborn arm uses takeup_rate; the prenatal
arm uses takeup_rate × PRENATAL_TAKEUP_RATIO (0.92, the Flint 0.90/0.98 ratio).
The library default leaves the arms uniform (backward compatible); the forecast
applies the split. The band scales prenatal with the swept postnatal rate.

A nice property: the Flint scenario (--takeup-rate 0.98) yields 0.98/0.90 —
recovering Flint's observed arm rates exactly.

Effect: conservative headline $54.4M -> $52.9M (prenatal arm scaled to 0.83;
postnatal unchanged); Flint $65M -> $63M. Recipients now correctly differ by
arm (~11,100 prenatal vs ~12,100 infants). Adds a test; full suite 1559 pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
+++ b/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>54399559.50000001</v>
+        <v>52948904.58000001</v>
       </c>
     </row>
     <row r="6">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>18133186.5</v>
+        <v>16682531.58</v>
       </c>
     </row>
     <row r="7">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>50035359.45905797</v>
+        <v>48701083.20681643</v>
       </c>
     </row>
     <row r="9">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>58763759.54094204</v>
+        <v>57196725.95318358</v>
       </c>
     </row>
     <row r="10">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>2653009.14342981</v>
+        <v>2582262.232938347</v>
       </c>
     </row>
     <row r="11">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32639735.70000001</v>
+        <v>31769342.74800001</v>
       </c>
     </row>
     <row r="12">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>69359438.3625</v>
+        <v>67510860.73875001</v>
       </c>
     </row>
     <row r="13">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>36266372.99999999</v>
+        <v>36266373.00000001</v>
       </c>
     </row>
     <row r="16">
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>90665932.5</v>
+        <v>89215277.58000001</v>
       </c>
     </row>
     <row r="17">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>22750433.0625</v>
+        <v>21964661.6475</v>
       </c>
     </row>
     <row r="20">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>9822142.687500002</v>
+        <v>9036371.272500001</v>
       </c>
     </row>
     <row r="21">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>41.8</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="24">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>35510823.5625</v>
+        <v>34362388.4175</v>
       </c>
     </row>
     <row r="25">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>15166955.375</v>
+        <v>14643107.765</v>
       </c>
     </row>
     <row r="26">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>24177.582</v>
+        <v>23210.47872</v>
       </c>
     </row>
     <row r="30">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>12088.791</v>
+        <v>11121.68772</v>
       </c>
     </row>
     <row r="31">
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>2250</v>
+        <v>2281.25</v>
       </c>
     </row>
     <row r="33">
@@ -852,13 +852,13 @@
         <v>109745</v>
       </c>
       <c r="D2" s="11" t="n">
-        <v>4377</v>
+        <v>4202</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>9847867</v>
+        <v>9585257</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>2250</v>
+        <v>2281</v>
       </c>
       <c r="G2" s="12" t="n">
         <v>18.1</v>
@@ -877,13 +877,13 @@
         <v>109845</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>6017</v>
+        <v>5776</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>13537408</v>
+        <v>13176411</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>2250</v>
+        <v>2281</v>
       </c>
       <c r="G3" s="12" t="n">
         <v>24.9</v>
@@ -902,13 +902,13 @@
         <v>109868</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>6596</v>
+        <v>6333</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>14842100</v>
+        <v>14446310</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>2250</v>
+        <v>2281</v>
       </c>
       <c r="G4" s="12" t="n">
         <v>27.3</v>
@@ -927,13 +927,13 @@
         <v>109862</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>4232</v>
+        <v>4063</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>9523097</v>
+        <v>9269148</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>2250</v>
+        <v>2281</v>
       </c>
       <c r="G5" s="12" t="n">
         <v>17.5</v>
@@ -952,13 +952,13 @@
         <v>109855</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>2955</v>
+        <v>2837</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>6649088</v>
+        <v>6471779</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>2250</v>
+        <v>2281</v>
       </c>
       <c r="G6" s="12" t="n">
         <v>12.2</v>
@@ -1025,19 +1025,19 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>10240530</v>
+        <v>9967449</v>
       </c>
       <c r="C2" s="11" t="n">
-        <v>3413510</v>
+        <v>3140429</v>
       </c>
       <c r="D2" s="11" t="n">
         <v>6827020</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>1192171</v>
+        <v>1160380</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>4551</v>
+        <v>4369</v>
       </c>
     </row>
     <row r="3">
@@ -1047,19 +1047,19 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>35883688</v>
+        <v>34926790</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>11961230</v>
+        <v>11004331</v>
       </c>
       <c r="D3" s="11" t="n">
         <v>23922459</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>2109491</v>
+        <v>2053238</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>15948</v>
+        <v>15310</v>
       </c>
     </row>
     <row r="4">
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>2244518</v>
+        <v>2184664</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>748173</v>
+        <v>688319</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>1496345</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>514832</v>
+        <v>501103</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>998</v>
+        <v>958</v>
       </c>
     </row>
     <row r="5">
@@ -1091,19 +1091,19 @@
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>6030823</v>
+        <v>5870001</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>2010274</v>
+        <v>1849452</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>4020548</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>838695</v>
+        <v>816330</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>2680</v>
+        <v>2573</v>
       </c>
     </row>
   </sheetData>
@@ -1117,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1213,7 +1213,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Take-up rate</t>
+          <t>Take-up — postnatal (newborn)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1221,120 +1221,135 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Combined eligibility×claim (Flint observed 0.98); swept for the band</t>
+          <t>Flint observed 0.98; swept for the band</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fertility response</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>+0%</t>
-        </is>
+          <t>Take-up — prenatal</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.828</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Induced eligible-birth increase (Flint ~+10%); scales both arms</t>
+          <t>0.92× postnatal (Flint: ~90% prenatal vs 98% newborn)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Birth rate / dependent</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.066</v>
+          <t>Fertility response</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>+0%</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Annual births ÷ dependents (FLOW); drives both arms; swept ±25%</t>
+          <t>Induced eligible-birth increase (Flint ~+10%); scales both arms</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pregnancy Medicaid pathway</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1.96× FPL</t>
-        </is>
+          <t>Birth rate / dependent</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.066</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Clause 1 prenatal pathway (196% FPL); subsumed by the 300% income test</t>
+          <t>Annual births ÷ dependents (FLOW); drives both arms; swept ±25%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FPL table year</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>2028</v>
+          <t>Pregnancy Medicaid pathway</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1.96× FPL</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>benefits/_fpl.py (2025 published; 2026-28 CPI-projected)</t>
+          <t>Clause 1 prenatal pathway (196% FPL); subsumed by the 300% income test</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tax treatment</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>non-taxable</t>
-        </is>
+          <t>FPL table year</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2028</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Added to SPM resources only; no AGI/EITC/CTC interaction</t>
+          <t>benefits/_fpl.py (2025 published; 2026-28 CPI-projected)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fiscal weight</t>
+          <t>Tax treatment</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>WGTP (household)</t>
+          <t>non-taxable</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SPM-grain household weight; not the EITC-reweighted tax-unit weight</t>
+          <t>Added to SPM resources only; no AGI/EITC/CTC interaction</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Fiscal weight</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>WGTP (household)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SPM-grain household weight; not the EITC-reweighted tax-unit weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Income quintiles</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>WGTP-weighted</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>SPM units ranked on summed income; population-equal fifths</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): regenerate rxkids_2028 reports against 2026-07-05 refresh
Re-run forecast_rxkids_2028.py (tax-year 2028, all 3 scenarios) against
the freshly merged monthly anchor/panel data. Topline costs, county, and
state breakdowns are unchanged; only rounding-level quintile family-count
noise and binary metadata shifted. Full suite green (1604 passed, 3 skipped).
</commit_message>
<xml_diff>
--- a/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
+++ b/reports/rxkids_2028/rxkids_2028_cost_and_impact.xlsx
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>7326.023534804361</v>
+        <v>7326.02353480436</v>
       </c>
     </row>
     <row r="34">
@@ -871,7 +871,7 @@
         <v>15315</v>
       </c>
       <c r="C2" s="11" t="n">
-        <v>107149</v>
+        <v>107150</v>
       </c>
       <c r="D2" s="11" t="n">
         <v>2230</v>
@@ -896,7 +896,7 @@
         <v>52619</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>107150</v>
+        <v>107149</v>
       </c>
       <c r="D3" s="11" t="n">
         <v>4377</v>

</xml_diff>